<commit_message>
Need to check participant 019 s l3, l4 beta
</commit_message>
<xml_diff>
--- a/002_AEROTEX_IHB3D/gridConvergence_D01_V1.xlsx
+++ b/002_AEROTEX_IHB3D/gridConvergence_D01_V1.xlsx
@@ -13110,6 +13110,7 @@
   <mergeCells count="18">
     <mergeCell ref="A25:I25"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="D37:F37"/>
     <mergeCell ref="A37:C37"/>
     <mergeCell ref="G37:I37"/>
@@ -13121,10 +13122,9 @@
     <mergeCell ref="D26:F26"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="G26:I26"/>
-    <mergeCell ref="D15:F15"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="D15:F15"/>
     <mergeCell ref="G15:I15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13187,13 +13187,13 @@
         <v>0</v>
       </c>
       <c r="B3" s="11" t="n">
-        <v>0.4584</v>
+        <v>0.43714</v>
       </c>
       <c r="C3" s="11" t="n">
-        <v>0.0106</v>
+        <v>0.01008</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>-0.0007</v>
+        <v>-0.0006400000000000001</v>
       </c>
       <c r="E3" s="10" t="n"/>
       <c r="F3" s="10" t="n"/>
@@ -14271,10 +14271,10 @@
         <v>0</v>
       </c>
       <c r="B6" s="11" t="n">
-        <v>0.4597</v>
+        <v>0.43858</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>0.0107</v>
+        <v>0.01019</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>-0.001</v>
@@ -15355,13 +15355,13 @@
         <v>0</v>
       </c>
       <c r="B9" s="39" t="n">
-        <v>0.4676</v>
+        <v>0.44616</v>
       </c>
       <c r="C9" s="39" t="n">
-        <v>0.0114</v>
+        <v>0.0109</v>
       </c>
       <c r="D9" s="39" t="n">
-        <v>-0.0031</v>
+        <v>-0.00292</v>
       </c>
       <c r="E9" s="10" t="n"/>
       <c r="F9" s="10" t="n"/>
@@ -16436,13 +16436,13 @@
         <v>0</v>
       </c>
       <c r="B12" s="11" t="n">
-        <v>0.4607</v>
+        <v>0.43954</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>0.0125</v>
+        <v>0.01194</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>-0.002</v>
+        <v>-0.00189</v>
       </c>
       <c r="E12" s="10" t="n"/>
       <c r="F12" s="10" t="n"/>

</xml_diff>